<commit_message>
Update lead template workbook
Refresh the lead template Excel workbook to include the latest template revisions for lead data capture.
</commit_message>
<xml_diff>
--- a/outputs/260908-2225-lead-template/lead-template.xlsx
+++ b/outputs/260908-2225-lead-template/lead-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\CRM\frappe-crm\outputs\260908-2225-lead-template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2CB8129-D882-4CB8-A435-4B8568629FD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0A6F440-2D59-4035-88B2-45B4BCF668C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="16080" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lead Template" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="76">
   <si>
     <t>Họ và tên</t>
   </si>
@@ -161,36 +161,15 @@
     <t>0912345678</t>
   </si>
   <si>
-    <t>Hà Nội</t>
-  </si>
-  <si>
-    <t>THPT Chu Văn An</t>
-  </si>
-  <si>
-    <t>Facebook</t>
-  </si>
-  <si>
     <t>Quan tâm ngành Marketing.</t>
   </si>
   <si>
-    <t>Digital Marketing</t>
-  </si>
-  <si>
     <t>Lê Văn Cường</t>
   </si>
   <si>
     <t>0923456789</t>
   </si>
   <si>
-    <t>Đà Nẵng</t>
-  </si>
-  <si>
-    <t>THPT Phan Châu Trinh</t>
-  </si>
-  <si>
-    <t>Zalo</t>
-  </si>
-  <si>
     <t>Muốn tìm hiểu học bổng.</t>
   </si>
   <si>
@@ -200,139 +179,73 @@
     <t>0934567890</t>
   </si>
   <si>
-    <t>Cần Thơ</t>
-  </si>
-  <si>
-    <t>THPT Châu Văn Liêm</t>
-  </si>
-  <si>
-    <t>Website</t>
-  </si>
-  <si>
     <t>Nguyện vọng 2</t>
   </si>
   <si>
     <t>Quan tâm ngành Thiết kế đồ họa.</t>
   </si>
   <si>
-    <t>Graphic Design</t>
-  </si>
-  <si>
     <t>Hoàng Văn Em</t>
   </si>
   <si>
     <t>0945678901</t>
   </si>
   <si>
-    <t>Hải Phòng</t>
-  </si>
-  <si>
-    <t>THPT Ngô Quyền</t>
-  </si>
-  <si>
     <t>Quan tâm chương trình học bổng tài năng.</t>
   </si>
   <si>
-    <t>Business Administration</t>
-  </si>
-  <si>
     <t>Vũ Thị Giang</t>
   </si>
   <si>
     <t>0956789012</t>
   </si>
   <si>
-    <t>THPT Lê Hồng Phong</t>
-  </si>
-  <si>
     <t>Quan tâm ngành Trí tuệ nhân tạo.</t>
   </si>
   <si>
-    <t>Artificial Intelligence</t>
-  </si>
-  <si>
     <t>Đặng Văn Hùng</t>
   </si>
   <si>
     <t>0967890123</t>
   </si>
   <si>
-    <t>Bình Dương</t>
-  </si>
-  <si>
-    <t>THPT Trịnh Hoài Đức</t>
-  </si>
-  <si>
     <t>Muốn biết thông tin học phí.</t>
   </si>
   <si>
-    <t>Information Assurance</t>
-  </si>
-  <si>
     <t>Bùi Thị Kim</t>
   </si>
   <si>
     <t>0978901234</t>
   </si>
   <si>
-    <t>Đồng Nai</t>
-  </si>
-  <si>
     <t>Quan tâm ngành Quản trị khách sạn.</t>
   </si>
   <si>
-    <t>Hospitality Management</t>
-  </si>
-  <si>
     <t>Ngô Văn Long</t>
   </si>
   <si>
     <t>0989012345</t>
   </si>
   <si>
-    <t>Khánh Hòa</t>
-  </si>
-  <si>
-    <t>THPT Lý Tự Trọng</t>
-  </si>
-  <si>
     <t>Quan tâm chương trình đào tạo song ngữ.</t>
   </si>
   <si>
-    <t>International Business</t>
-  </si>
-  <si>
     <t>Trịnh Thị Mai</t>
   </si>
   <si>
     <t>0990123456</t>
   </si>
   <si>
-    <t>Thừa Thiên Huế</t>
-  </si>
-  <si>
-    <t>THPT Quốc Học</t>
-  </si>
-  <si>
     <t>Nguyện vọng 3</t>
   </si>
   <si>
     <t>Quan tâm ngành Truyền thông đa phương tiện.</t>
   </si>
   <si>
-    <t>Multimedia Communications</t>
-  </si>
-  <si>
     <t>Phan Văn Nam</t>
   </si>
   <si>
     <t>0901122334</t>
-  </si>
-  <si>
-    <t>An Giang</t>
-  </si>
-  <si>
-    <t>THPT Long Xuyên</t>
   </si>
   <si>
     <t>Quan tâm học bổng Nguyễn Văn Đạo.</t>
@@ -989,56 +902,56 @@
         <v>45</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="J6" s="15">
         <v>2026</v>
       </c>
       <c r="K6" s="22" t="s">
-        <v>50</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="6" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>53</v>
+        <v>13</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>54</v>
+        <v>14</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>55</v>
+        <v>16</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="J7" s="15">
         <v>2026</v>
@@ -1049,49 +962,49 @@
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="6" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>61</v>
+        <v>16</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="J8" s="15">
         <v>2026</v>
       </c>
       <c r="K8" s="22" t="s">
-        <v>64</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="6" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>67</v>
+        <v>13</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>68</v>
+        <v>14</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>15</v>
@@ -1104,126 +1017,126 @@
         <v>17</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="J9" s="15">
         <v>2026</v>
       </c>
       <c r="K9" s="22" t="s">
-        <v>70</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="6" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>73</v>
+        <v>14</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="J10" s="15">
         <v>2026</v>
       </c>
       <c r="K10" s="22" t="s">
-        <v>75</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="6" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>78</v>
+        <v>13</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>79</v>
+        <v>14</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>55</v>
+        <v>16</v>
       </c>
       <c r="G11" s="2"/>
       <c r="H11" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I11" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>80</v>
       </c>
       <c r="J11" s="15">
         <v>2026</v>
       </c>
       <c r="K11" s="22" t="s">
-        <v>81</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="6" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>83</v>
+        <v>64</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>84</v>
+        <v>13</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>68</v>
+        <v>14</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>61</v>
+        <v>16</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="J12" s="15">
         <v>2026</v>
       </c>
       <c r="K12" s="22" t="s">
-        <v>86</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="6" t="s">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>88</v>
+        <v>67</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>89</v>
+        <v>13</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>90</v>
+        <v>14</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>15</v>
@@ -1236,73 +1149,73 @@
         <v>17</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="J13" s="15">
         <v>2026</v>
       </c>
       <c r="K13" s="22" t="s">
-        <v>92</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="6" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>95</v>
+        <v>13</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>96</v>
+        <v>14</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="G14" s="2"/>
       <c r="H14" s="2" t="s">
-        <v>97</v>
+        <v>71</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>98</v>
+        <v>72</v>
       </c>
       <c r="J14" s="15">
         <v>2026</v>
       </c>
       <c r="K14" s="22" t="s">
-        <v>99</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="6" t="s">
-        <v>100</v>
+        <v>73</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>101</v>
+        <v>74</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>102</v>
+        <v>13</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>103</v>
+        <v>14</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>55</v>
+        <v>16</v>
       </c>
       <c r="G15" s="2"/>
       <c r="H15" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>104</v>
+        <v>75</v>
       </c>
       <c r="J15" s="15">
         <v>2026</v>

</xml_diff>